<commit_message>
Remove ACC I from AZ BAU
</commit_message>
<xml_diff>
--- a/InputData/trans/BRZSPbS/BAU Required ZEV Sales Perc by Subregion.xlsx
+++ b/InputData/trans/BRZSPbS/BAU Required ZEV Sales Perc by Subregion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-maryland\InputData\trans\BRZSPbS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-arizona\InputData\trans\BRZSPbS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBC4FF3-5DA9-4781-AF0A-8E522124D4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C89409-4E12-410B-BB32-ADE81A9BCE39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29235" yWindow="3030" windowWidth="17505" windowHeight="9735" firstSheet="2" activeTab="3" xr2:uid="{8F1AFB95-7E48-4A2A-86D9-67ED7638AFF8}"/>
+    <workbookView xWindow="58830" yWindow="2520" windowWidth="23085" windowHeight="13305" firstSheet="2" activeTab="3" xr2:uid="{8F1AFB95-7E48-4A2A-86D9-67ED7638AFF8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -6855,128 +6855,97 @@
         <v>143</v>
       </c>
       <c r="B2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=B$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!B$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!B$2),0)</f>
-        <v>9.5000000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=C$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!C$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!C$2),0)</f>
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=D$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!D$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!D$2),0)</f>
-        <v>0.14499999999999999</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=E$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!E$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!E$2),0)</f>
-        <v>0.16999999999999998</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=F$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!F$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!F$2),0)</f>
-        <v>0.19500000000000001</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=G$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!G$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!G$2),0)</f>
-        <v>0.21999999999999997</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=H$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!H$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!H$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=I$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!I$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!I$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=J$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!J$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!J$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=K$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!K$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!K$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=L$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!L$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!L$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=M$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!M$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!M$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=N$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!N$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!N$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=O$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!O$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!O$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=P$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!P$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!P$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=Q$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!Q$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!Q$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=R$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!R$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!R$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=S$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!S$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!S$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=T$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!T$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!T$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="U2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=U$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!U$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!U$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="V2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=V$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!V$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!V$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="W2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=W$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!W$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!W$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=X$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!X$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!X$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="Y2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=Y$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!Y$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!Y$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=Z$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!Z$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!Z$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=AA$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!AA$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!AA$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AB2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=AB$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!AB$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!AB$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AC2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=AC$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!AC$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!AC$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AD2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=AD$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!AD$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!AD$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AE2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=AE$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!AE$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!AE$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AF2">
-        <f>IF(INDEX('CA Standards and Followers'!$E$13:$E$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))&lt;=AF$1,IF(INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))=1,'CA Standards and Followers'!AF$3*INDEX('CA Standards and Followers'!$C$13:$C$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0)),INDEX('CA Standards and Followers'!$B$13:$B$72,MATCH($A2,'CA Standards and Followers'!$A$13:$A$72,0))*'CA Standards and Followers'!AF$2),0)</f>
-        <v>0.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.35">

</xml_diff>